<commit_message>
Further work on UKWA analysis - fix links to results.weymouthspeedweek.com
</commit_message>
<xml_diff>
--- a/resources/ukwa/analysis/percentiles.xlsx
+++ b/resources/ukwa/analysis/percentiles.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26924"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\mike\projects\work\wsw-results\resources\ukwa\analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64E297EC-12FA-4F30-9052-8137B0C04C61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3504CC08-34C9-49E4-9C9E-84361A9724B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{BC2B614C-97CE-4BFB-A796-CE0AF2755093}"/>
   </bookViews>
@@ -17,6 +17,16 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$G$117</definedName>
+    <definedName name="_xlchart.v1.0" hidden="1">Sheet1!$C$1</definedName>
+    <definedName name="_xlchart.v1.1" hidden="1">Sheet1!$C$2:$C$124</definedName>
+    <definedName name="_xlchart.v1.2" hidden="1">Sheet1!$D$1</definedName>
+    <definedName name="_xlchart.v1.3" hidden="1">Sheet1!$D$2:$D$124</definedName>
+    <definedName name="_xlchart.v1.4" hidden="1">Sheet1!$D$1</definedName>
+    <definedName name="_xlchart.v1.5" hidden="1">Sheet1!$D$2:$D$124</definedName>
+    <definedName name="_xlchart.v1.6" hidden="1">Sheet1!$D$1</definedName>
+    <definedName name="_xlchart.v1.7" hidden="1">Sheet1!$D$2:$D$124</definedName>
+    <definedName name="_xlchart.v1.8" hidden="1">Sheet1!$D$1</definedName>
+    <definedName name="_xlchart.v1.9" hidden="1">Sheet1!$D$2:$D$124</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -3455,6 +3465,146 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chartEx1.xml><?xml version="1.0" encoding="utf-8"?>
+<cx:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex">
+  <cx:chartData>
+    <cx:data id="0">
+      <cx:numDim type="val">
+        <cx:f>_xlchart.v1.5</cx:f>
+      </cx:numDim>
+    </cx:data>
+  </cx:chartData>
+  <cx:chart>
+    <cx:title pos="t" align="ctr" overlay="0">
+      <cx:tx>
+        <cx:txData>
+          <cx:v>Median Times for UKWA - 2010 to 2023</cx:v>
+        </cx:txData>
+      </cx:tx>
+      <cx:txPr>
+        <a:bodyPr spcFirstLastPara="1" vertOverflow="ellipsis" horzOverflow="overflow" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr" rtl="0">
+            <a:defRPr/>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="en-US" sz="1400" b="0" i="0" u="none" strike="noStrike" baseline="0">
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:sysClr>
+              </a:solidFill>
+              <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+            </a:rPr>
+            <a:t>Median Times for UKWA - 2010 to 2023</a:t>
+          </a:r>
+        </a:p>
+      </cx:txPr>
+    </cx:title>
+    <cx:plotArea>
+      <cx:plotAreaRegion>
+        <cx:series layoutId="clusteredColumn" uniqueId="{0C3C6711-4380-4A2A-9B4F-25CBC4A6D851}">
+          <cx:tx>
+            <cx:txData>
+              <cx:f>_xlchart.v1.4</cx:f>
+              <cx:v>median</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:dataId val="0"/>
+          <cx:layoutPr>
+            <cx:binning intervalClosed="r">
+              <cx:binCount val="12"/>
+            </cx:binning>
+          </cx:layoutPr>
+        </cx:series>
+      </cx:plotAreaRegion>
+      <cx:axis id="0">
+        <cx:catScaling gapWidth="0"/>
+        <cx:tickLabels/>
+        <cx:numFmt formatCode="0.0" sourceLinked="0"/>
+      </cx:axis>
+      <cx:axis id="1">
+        <cx:valScaling/>
+        <cx:majorGridlines/>
+        <cx:tickLabels/>
+      </cx:axis>
+    </cx:plotArea>
+  </cx:chart>
+</cx:chartSpace>
+</file>
+
+<file path=xl/charts/chartEx2.xml><?xml version="1.0" encoding="utf-8"?>
+<cx:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex">
+  <cx:chartData>
+    <cx:data id="0">
+      <cx:numDim type="val">
+        <cx:f>_xlchart.v1.1</cx:f>
+      </cx:numDim>
+    </cx:data>
+  </cx:chartData>
+  <cx:chart>
+    <cx:title pos="t" align="ctr" overlay="0">
+      <cx:tx>
+        <cx:txData>
+          <cx:v>25th Percentile for UKWA - 2010 to 2023</cx:v>
+        </cx:txData>
+      </cx:tx>
+      <cx:txPr>
+        <a:bodyPr spcFirstLastPara="1" vertOverflow="ellipsis" horzOverflow="overflow" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr" rtl="0">
+            <a:defRPr/>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="en-US" sz="1400" b="0" i="0" u="none" strike="noStrike" baseline="0">
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:sysClr>
+              </a:solidFill>
+              <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+            </a:rPr>
+            <a:t>25th Percentile for UKWA - 2010 to 2023</a:t>
+          </a:r>
+        </a:p>
+      </cx:txPr>
+    </cx:title>
+    <cx:plotArea>
+      <cx:plotAreaRegion>
+        <cx:series layoutId="clusteredColumn" uniqueId="{0C3C6711-4380-4A2A-9B4F-25CBC4A6D851}">
+          <cx:tx>
+            <cx:txData>
+              <cx:f>_xlchart.v1.0</cx:f>
+              <cx:v>25th percentile</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:dataId val="0"/>
+          <cx:layoutPr>
+            <cx:binning intervalClosed="r">
+              <cx:binCount val="12"/>
+            </cx:binning>
+          </cx:layoutPr>
+        </cx:series>
+      </cx:plotAreaRegion>
+      <cx:axis id="0">
+        <cx:catScaling gapWidth="0"/>
+        <cx:tickLabels/>
+        <cx:numFmt formatCode="0.0" sourceLinked="0"/>
+      </cx:axis>
+      <cx:axis id="1">
+        <cx:valScaling/>
+        <cx:majorGridlines/>
+        <cx:tickLabels/>
+      </cx:axis>
+    </cx:plotArea>
+  </cx:chart>
+</cx:chartSpace>
+</file>
+
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
@@ -3575,6 +3725,86 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors4.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors5.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
@@ -5106,6 +5336,1022 @@
         <a:noFill/>
       </a:ln>
     </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style4.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="366">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat">
+        <a:solidFill>
+          <a:srgbClr val="D9D9D9"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDash"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style5.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="366">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat">
+        <a:solidFill>
+          <a:srgbClr val="D9D9D9"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDash"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
   </cs:wall>
 </cs:chartStyle>
 </file>
@@ -5226,13 +6472,169 @@
     </xdr:graphicFrame>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>609599</xdr:colOff>
+      <xdr:row>71</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>25</xdr:col>
+      <xdr:colOff>600074</xdr:colOff>
+      <xdr:row>90</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" Requires="cx1">
+        <xdr:graphicFrame macro="">
+          <xdr:nvGraphicFramePr>
+            <xdr:cNvPr id="4" name="Chart 3">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9B1D035B-81A2-4CA4-9AFF-FD1488D4A96B}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvGraphicFramePr/>
+          </xdr:nvGraphicFramePr>
+          <xdr:xfrm>
+            <a:off x="0" y="0"/>
+            <a:ext cx="0" cy="0"/>
+          </xdr:xfrm>
+          <a:graphic>
+            <a:graphicData uri="http://schemas.microsoft.com/office/drawing/2014/chartex">
+              <cx:chart xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+            </a:graphicData>
+          </a:graphic>
+        </xdr:graphicFrame>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="0" name=""/>
+            <xdr:cNvSpPr>
+              <a:spLocks noTextEdit="1"/>
+            </xdr:cNvSpPr>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="10801349" y="13525500"/>
+              <a:ext cx="6696075" cy="3695700"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:solidFill>
+              <a:prstClr val="white"/>
+            </a:solidFill>
+            <a:ln w="1">
+              <a:solidFill>
+                <a:prstClr val="green"/>
+              </a:solidFill>
+            </a:ln>
+          </xdr:spPr>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" horzOverflow="clip"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:r>
+                <a:rPr lang="en-GB" sz="1100"/>
+                <a:t>This chart isn't available in your version of Excel.
+Editing this shape or saving this workbook into a different file format will permanently break the chart.</a:t>
+              </a:r>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>92</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>25</xdr:col>
+      <xdr:colOff>600075</xdr:colOff>
+      <xdr:row>111</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" Requires="cx1">
+        <xdr:graphicFrame macro="">
+          <xdr:nvGraphicFramePr>
+            <xdr:cNvPr id="5" name="Chart 4">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8BCEF1ED-E10B-471F-A37F-792DD58CD3C5}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvGraphicFramePr/>
+          </xdr:nvGraphicFramePr>
+          <xdr:xfrm>
+            <a:off x="0" y="0"/>
+            <a:ext cx="0" cy="0"/>
+          </xdr:xfrm>
+          <a:graphic>
+            <a:graphicData uri="http://schemas.microsoft.com/office/drawing/2014/chartex">
+              <cx:chart xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
+            </a:graphicData>
+          </a:graphic>
+        </xdr:graphicFrame>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="0" name=""/>
+            <xdr:cNvSpPr>
+              <a:spLocks noTextEdit="1"/>
+            </xdr:cNvSpPr>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="10801350" y="17526000"/>
+              <a:ext cx="6696075" cy="3695700"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:solidFill>
+              <a:prstClr val="white"/>
+            </a:solidFill>
+            <a:ln w="1">
+              <a:solidFill>
+                <a:prstClr val="green"/>
+              </a:solidFill>
+            </a:ln>
+          </xdr:spPr>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" horzOverflow="clip"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:r>
+                <a:rPr lang="en-GB" sz="1100"/>
+                <a:t>This chart isn't available in your version of Excel.
+Editing this shape or saving this workbook into a different file format will permanently break the chart.</a:t>
+              </a:r>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -5270,7 +6672,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -5376,7 +6778,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -5518,7 +6920,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>

</xml_diff>

<commit_message>
Add r-squared to analysis
</commit_message>
<xml_diff>
--- a/resources/ukwa/analysis/percentiles.xlsx
+++ b/resources/ukwa/analysis/percentiles.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\mike\projects\work\wsw-results\resources\ukwa\analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3504CC08-34C9-49E4-9C9E-84361A9724B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52451064-4A49-46B2-86B9-1A2EEFA310EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{BC2B614C-97CE-4BFB-A796-CE0AF2755093}"/>
   </bookViews>
@@ -21,12 +21,6 @@
     <definedName name="_xlchart.v1.1" hidden="1">Sheet1!$C$2:$C$124</definedName>
     <definedName name="_xlchart.v1.2" hidden="1">Sheet1!$D$1</definedName>
     <definedName name="_xlchart.v1.3" hidden="1">Sheet1!$D$2:$D$124</definedName>
-    <definedName name="_xlchart.v1.4" hidden="1">Sheet1!$D$1</definedName>
-    <definedName name="_xlchart.v1.5" hidden="1">Sheet1!$D$2:$D$124</definedName>
-    <definedName name="_xlchart.v1.6" hidden="1">Sheet1!$D$1</definedName>
-    <definedName name="_xlchart.v1.7" hidden="1">Sheet1!$D$2:$D$124</definedName>
-    <definedName name="_xlchart.v1.8" hidden="1">Sheet1!$D$1</definedName>
-    <definedName name="_xlchart.v1.9" hidden="1">Sheet1!$D$2:$D$124</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -326,8 +320,44 @@
               <a:effectLst/>
             </c:spPr>
             <c:trendlineType val="linear"/>
-            <c:dispRSqr val="0"/>
+            <c:dispRSqr val="1"/>
             <c:dispEq val="0"/>
+            <c:trendlineLbl>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="-7.4241989478718323E-2"/>
+                  <c:y val="8.4399541121386971E-3"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:numFmt formatCode="General" sourceLinked="0"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="65000"/>
+                          <a:lumOff val="35000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:latin typeface="+mn-lt"/>
+                      <a:ea typeface="+mn-ea"/>
+                      <a:cs typeface="+mn-cs"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="en-US"/>
+                </a:p>
+              </c:txPr>
+            </c:trendlineLbl>
           </c:trendline>
           <c:xVal>
             <c:numRef>
@@ -1462,8 +1492,44 @@
               <a:effectLst/>
             </c:spPr>
             <c:trendlineType val="linear"/>
-            <c:dispRSqr val="0"/>
+            <c:dispRSqr val="1"/>
             <c:dispEq val="0"/>
+            <c:trendlineLbl>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="-0.18406504065040649"/>
+                  <c:y val="2.0411520228647485E-2"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:numFmt formatCode="General" sourceLinked="0"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="65000"/>
+                          <a:lumOff val="35000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:latin typeface="+mn-lt"/>
+                      <a:ea typeface="+mn-ea"/>
+                      <a:cs typeface="+mn-cs"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="en-US"/>
+                </a:p>
+              </c:txPr>
+            </c:trendlineLbl>
           </c:trendline>
           <c:xVal>
             <c:numRef>
@@ -3470,7 +3536,7 @@
   <cx:chartData>
     <cx:data id="0">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.5</cx:f>
+        <cx:f>_xlchart.v1.3</cx:f>
       </cx:numDim>
     </cx:data>
   </cx:chartData>
@@ -3508,7 +3574,7 @@
         <cx:series layoutId="clusteredColumn" uniqueId="{0C3C6711-4380-4A2A-9B4F-25CBC4A6D851}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.4</cx:f>
+              <cx:f>_xlchart.v1.2</cx:f>
               <cx:v>median</cx:v>
             </cx:txData>
           </cx:tx>

</xml_diff>